<commit_message>
Fitbit-Tabelle rechnet ihre Groesse statt sie abzutasten
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/skin/Skin-Matrix.xlsx
+++ b/docs/skin/Skin-Matrix.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Matrix" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$H$390</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Matrix'!$A$1:$H$395</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H390"/>
+  <dimension ref="A1:H395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -11611,19 +11611,15 @@
           <t>Statistik</t>
         </is>
       </c>
-      <c r="C297" t="inlineStr">
-        <is>
-          <t>:focused</t>
-        </is>
-      </c>
+      <c r="C297" t="inlineStr"/>
       <c r="D297" t="inlineStr">
         <is>
-          <t>.my-table-view:focused</t>
+          <t>.my-table-view .text-field</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-background-insets</t>
         </is>
       </c>
       <c r="F297" t="inlineStr">
@@ -11638,7 +11634,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>"-fx-control-inner-background"</t>
+          <t>"0"</t>
         </is>
       </c>
     </row>
@@ -11653,19 +11649,15 @@
           <t>Statistik</t>
         </is>
       </c>
-      <c r="C298" t="inlineStr">
-        <is>
-          <t>:focused</t>
-        </is>
-      </c>
+      <c r="C298" t="inlineStr"/>
       <c r="D298" t="inlineStr">
         <is>
-          <t>.my-table-view:focused</t>
+          <t>.my-table-view .text-field</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>-fx-background-insets</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F298" t="inlineStr">
@@ -11695,14 +11687,10 @@
           <t>Statistik</t>
         </is>
       </c>
-      <c r="C299" t="inlineStr">
-        <is>
-          <t>:focused</t>
-        </is>
-      </c>
+      <c r="C299" t="inlineStr"/>
       <c r="D299" t="inlineStr">
         <is>
-          <t>.my-table-view:focused</t>
+          <t>.my-table-view .text-field</t>
         </is>
       </c>
       <c r="E299" t="inlineStr">
@@ -11729,57 +11717,69 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Schlagwort — Löschknopf</t>
+          <t>Tabelle</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Tagebuch</t>
-        </is>
-      </c>
-      <c r="C300" t="inlineStr"/>
+          <t>Statistik</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>.tag-chip-remove</t>
+          <t>.my-table-view .text-field:focused</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-background-insets</t>
         </is>
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>playFieldBackground</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>← menuBarBackground</t>
-        </is>
-      </c>
-      <c r="H300" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>"0"</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Schlagwort — Löschknopf</t>
+          <t>Tabelle</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Tagebuch</t>
-        </is>
-      </c>
-      <c r="C301" t="inlineStr"/>
+          <t>Statistik</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>.tag-chip-remove</t>
+          <t>.my-table-view .text-field:focused</t>
         </is>
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>-fx-border-color</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
@@ -11794,30 +11794,34 @@
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>Color.TRANSPARENT</t>
+          <t>"0"</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Schlagwort — Löschknopf</t>
+          <t>Tabelle</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Tagebuch</t>
-        </is>
-      </c>
-      <c r="C302" t="inlineStr"/>
+          <t>Statistik</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>.tag-chip-remove</t>
+          <t>.my-table-view:focused</t>
         </is>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>-fx-border-width</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F302" t="inlineStr">
@@ -11832,30 +11836,34 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>"0px"</t>
+          <t>"-fx-control-inner-background"</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Schlagwort — Löschknopf</t>
+          <t>Tabelle</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Tagebuch</t>
-        </is>
-      </c>
-      <c r="C303" t="inlineStr"/>
+          <t>Statistik</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>.tag-chip-remove</t>
+          <t>.my-table-view:focused</t>
         </is>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>-fx-padding</t>
+          <t>-fx-background-insets</t>
         </is>
       </c>
       <c r="F303" t="inlineStr">
@@ -11870,48 +11878,56 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>"0 0"</t>
+          <t>"0"</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Schlagwort — Löschknopf</t>
+          <t>Tabelle</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Tagebuch</t>
-        </is>
-      </c>
-      <c r="C304" t="inlineStr"/>
+          <t>Statistik</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>.tag-chip-remove .text</t>
+          <t>.my-table-view:focused</t>
         </is>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>-fx-fill</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>textColor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H304" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>"0"</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Tagebuch — Layout</t>
+          <t>Schlagwort — Löschknopf</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -11922,34 +11938,30 @@
       <c r="C305" t="inlineStr"/>
       <c r="D305" t="inlineStr">
         <is>
-          <t>.diary-viewer-content</t>
+          <t>.tag-chip-remove</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>-fx-spacing</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>font</t>
+          <t>playFieldBackground</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H305" t="inlineStr">
-        <is>
-          <t>font.getSize() + "px"</t>
-        </is>
-      </c>
+          <t>← menuBarBackground</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Tagebuch — Layout</t>
+          <t>Schlagwort — Löschknopf</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -11960,34 +11972,34 @@
       <c r="C306" t="inlineStr"/>
       <c r="D306" t="inlineStr">
         <is>
-          <t>.diary-viewer-filter-bar</t>
+          <t>.tag-chip-remove</t>
         </is>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>-fx-max-width</t>
+          <t>-fx-border-color</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>diaryViewerContentWidth</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>fest im Code</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>diaryViewerContentWidth + "px"</t>
+          <t>Color.TRANSPARENT</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Tagebuch — Layout</t>
+          <t>Schlagwort — Löschknopf</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -11998,34 +12010,34 @@
       <c r="C307" t="inlineStr"/>
       <c r="D307" t="inlineStr">
         <is>
-          <t>.diary-viewer-filter-bar</t>
+          <t>.tag-chip-remove</t>
         </is>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>-fx-min-width</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>diaryViewerContentWidth</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>1200</t>
+          <t>fest im Code</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>diaryViewerContentWidth + "px"</t>
+          <t>"0px"</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Tagebuch — Layout</t>
+          <t>Schlagwort — Löschknopf</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -12036,30 +12048,34 @@
       <c r="C308" t="inlineStr"/>
       <c r="D308" t="inlineStr">
         <is>
-          <t>.diary-viewer-hint</t>
+          <t>.tag-chip-remove</t>
         </is>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>-fx-fill</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>incorrectTextColor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H308" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>"0 0"</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Tagebuch — Layout</t>
+          <t>Schlagwort — Löschknopf</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -12070,29 +12086,25 @@
       <c r="C309" t="inlineStr"/>
       <c r="D309" t="inlineStr">
         <is>
-          <t>.diary-viewer-hint</t>
+          <t>.tag-chip-remove .text</t>
         </is>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>-fx-font-style</t>
+          <t>-fx-fill</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>textColor</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>fest im Code</t>
-        </is>
-      </c>
-      <c r="H309" t="inlineStr">
-        <is>
-          <t>"italic"</t>
-        </is>
-      </c>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr"/>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -12108,12 +12120,12 @@
       <c r="C310" t="inlineStr"/>
       <c r="D310" t="inlineStr">
         <is>
-          <t>.diary-viewer-root</t>
+          <t>.diary-viewer-content</t>
         </is>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>-fx-padding</t>
+          <t>-fx-spacing</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -12128,7 +12140,7 @@
       </c>
       <c r="H310" t="inlineStr">
         <is>
-          <t>font.getSize() + "px 0px"</t>
+          <t>font.getSize() + "px"</t>
         </is>
       </c>
     </row>
@@ -12146,27 +12158,27 @@
       <c r="C311" t="inlineStr"/>
       <c r="D311" t="inlineStr">
         <is>
-          <t>.diary-viewer-scroll</t>
+          <t>.diary-viewer-filter-bar</t>
         </is>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>-fx-background</t>
+          <t>-fx-max-width</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>diaryViewerContentWidth</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>fest im Code</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>"transparent"</t>
+          <t>diaryViewerContentWidth + "px"</t>
         </is>
       </c>
     </row>
@@ -12184,27 +12196,27 @@
       <c r="C312" t="inlineStr"/>
       <c r="D312" t="inlineStr">
         <is>
-          <t>.diary-viewer-scroll</t>
+          <t>.diary-viewer-filter-bar</t>
         </is>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-min-width</t>
         </is>
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>diaryViewerContentWidth</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>fest im Code</t>
+          <t>1200</t>
         </is>
       </c>
       <c r="H312" t="inlineStr">
         <is>
-          <t>"transparent"</t>
+          <t>diaryViewerContentWidth + "px"</t>
         </is>
       </c>
     </row>
@@ -12222,17 +12234,17 @@
       <c r="C313" t="inlineStr"/>
       <c r="D313" t="inlineStr">
         <is>
-          <t>.diary-viewer-scroll</t>
+          <t>.diary-viewer-hint</t>
         </is>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>-fx-padding</t>
+          <t>-fx-fill</t>
         </is>
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t>font</t>
+          <t>incorrectTextColor</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
@@ -12240,11 +12252,7 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H313" t="inlineStr">
-        <is>
-          <t>"0 " + font.getSize() * 0.5 + "px 0 0"</t>
-        </is>
-      </c>
+      <c r="H313" t="inlineStr"/>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -12260,12 +12268,12 @@
       <c r="C314" t="inlineStr"/>
       <c r="D314" t="inlineStr">
         <is>
-          <t>.diary-viewer-scroll .viewport</t>
+          <t>.diary-viewer-hint</t>
         </is>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-font-style</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -12280,14 +12288,14 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>"transparent"</t>
+          <t>"italic"</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Tagebuchkarte</t>
+          <t>Tagebuch — Layout</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
@@ -12298,30 +12306,34 @@
       <c r="C315" t="inlineStr"/>
       <c r="D315" t="inlineStr">
         <is>
-          <t>.diary-card</t>
+          <t>.diary-viewer-root</t>
         </is>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t>displayTextQuestionBgColor</t>
+          <t>font</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>← displayTextBgColor</t>
-        </is>
-      </c>
-      <c r="H315" t="inlineStr"/>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>font.getSize() + "px 0px"</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Tagebuchkarte</t>
+          <t>Tagebuch — Layout</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
@@ -12332,34 +12344,34 @@
       <c r="C316" t="inlineStr"/>
       <c r="D316" t="inlineStr">
         <is>
-          <t>.diary-card</t>
+          <t>.diary-viewer-scroll</t>
         </is>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>-fx-background-insets</t>
+          <t>-fx-background</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>borderBigComponent</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>fest im Code</t>
         </is>
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>borderBigComponent.width() + "px"</t>
+          <t>"transparent"</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Tagebuchkarte</t>
+          <t>Tagebuch — Layout</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -12370,34 +12382,34 @@
       <c r="C317" t="inlineStr"/>
       <c r="D317" t="inlineStr">
         <is>
-          <t>.diary-card</t>
+          <t>.diary-viewer-scroll</t>
         </is>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>-fx-background-radius</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t>borderBigComponent</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>fest im Code</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>borderBigComponent.arc() + "px"</t>
+          <t>"transparent"</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Tagebuchkarte</t>
+          <t>Tagebuch — Layout</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -12408,17 +12420,17 @@
       <c r="C318" t="inlineStr"/>
       <c r="D318" t="inlineStr">
         <is>
-          <t>.diary-card</t>
+          <t>.diary-viewer-scroll</t>
         </is>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>-fx-border-color</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>borderBigComponent</t>
+          <t>font</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -12428,14 +12440,14 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>borderBigComponent.color()</t>
+          <t>"0 " + font.getSize() * 0.5 + "px 0 0"</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Tagebuchkarte</t>
+          <t>Tagebuch — Layout</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -12446,27 +12458,27 @@
       <c r="C319" t="inlineStr"/>
       <c r="D319" t="inlineStr">
         <is>
-          <t>.diary-card</t>
+          <t>.diary-viewer-scroll .viewport</t>
         </is>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>-fx-border-radius</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>borderBigComponent</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>fest im Code</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>borderBigComponent.arc() + "px"</t>
+          <t>"transparent"</t>
         </is>
       </c>
     </row>
@@ -12489,24 +12501,20 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>-fx-border-width</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>borderBigComponent</t>
+          <t>displayTextQuestionBgColor</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H320" t="inlineStr">
-        <is>
-          <t>borderBigComponent.width() + "px"</t>
-        </is>
-      </c>
+          <t>← displayTextBgColor</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -12527,22 +12535,22 @@
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>-fx-cursor</t>
+          <t>-fx-background-insets</t>
         </is>
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>borderBigComponent</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>fest im Code</t>
+          <t>Pflicht</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>"hand"</t>
+          <t>borderBigComponent.width() + "px"</t>
         </is>
       </c>
     </row>
@@ -12565,20 +12573,24 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>-fx-effect</t>
+          <t>-fx-background-radius</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>componentShadow</t>
+          <t>borderBigComponent</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>entfällt</t>
-        </is>
-      </c>
-      <c r="H322" t="inlineStr"/>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>borderBigComponent.arc() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -12599,12 +12611,12 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>-fx-padding</t>
+          <t>-fx-border-color</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>font</t>
+          <t>borderBigComponent</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
@@ -12614,7 +12626,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>font.getSize() + "px"</t>
+          <t>borderBigComponent.color()</t>
         </is>
       </c>
     </row>
@@ -12632,17 +12644,17 @@
       <c r="C324" t="inlineStr"/>
       <c r="D324" t="inlineStr">
         <is>
-          <t>.diary-card-date</t>
+          <t>.diary-card</t>
         </is>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>-fx-fill</t>
+          <t>-fx-border-radius</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>textColor</t>
+          <t>borderBigComponent</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -12650,7 +12662,11 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H324" t="inlineStr"/>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>borderBigComponent.arc() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -12666,27 +12682,27 @@
       <c r="C325" t="inlineStr"/>
       <c r="D325" t="inlineStr">
         <is>
-          <t>.diary-card-date</t>
+          <t>.diary-card</t>
         </is>
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>-fx-font-weight</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>borderBigComponent</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>fest im Code</t>
+          <t>Pflicht</t>
         </is>
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t>"bold"</t>
+          <t>borderBigComponent.width() + "px"</t>
         </is>
       </c>
     </row>
@@ -12704,25 +12720,29 @@
       <c r="C326" t="inlineStr"/>
       <c r="D326" t="inlineStr">
         <is>
-          <t>.diary-card-tags</t>
+          <t>.diary-card</t>
         </is>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>-fx-fill</t>
+          <t>-fx-cursor</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>textColor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H326" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>"hand"</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -12738,29 +12758,25 @@
       <c r="C327" t="inlineStr"/>
       <c r="D327" t="inlineStr">
         <is>
-          <t>.diary-card-tags</t>
+          <t>.diary-card</t>
         </is>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>-fx-font-style</t>
+          <t>-fx-effect</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>componentShadow</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>fest im Code</t>
-        </is>
-      </c>
-      <c r="H327" t="inlineStr">
-        <is>
-          <t>"italic"</t>
-        </is>
-      </c>
+          <t>entfällt</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -12776,17 +12792,17 @@
       <c r="C328" t="inlineStr"/>
       <c r="D328" t="inlineStr">
         <is>
-          <t>.diary-card-text</t>
+          <t>.diary-card</t>
         </is>
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>-fx-fill</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>textColor</t>
+          <t>font</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
@@ -12794,7 +12810,11 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H328" t="inlineStr"/>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>font.getSize() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -12807,29 +12827,25 @@
           <t>Tagebuch</t>
         </is>
       </c>
-      <c r="C329" t="inlineStr">
-        <is>
-          <t>:hover</t>
-        </is>
-      </c>
+      <c r="C329" t="inlineStr"/>
       <c r="D329" t="inlineStr">
         <is>
-          <t>.diary-card:hover</t>
+          <t>.diary-card-date</t>
         </is>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-fill</t>
         </is>
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>displayTextQuestionBgColor</t>
+          <t>textColor</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>← displayTextBgColor</t>
+          <t>Pflicht</t>
         </is>
       </c>
       <c r="H329" t="inlineStr"/>
@@ -12837,7 +12853,7 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Vorschlagsliste</t>
+          <t>Tagebuchkarte</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -12848,30 +12864,34 @@
       <c r="C330" t="inlineStr"/>
       <c r="D330" t="inlineStr">
         <is>
-          <t>.suggestion-box</t>
+          <t>.diary-card-date</t>
         </is>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-font-weight</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>menuBarBackground</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H330" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>"bold"</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Vorschlagsliste</t>
+          <t>Tagebuchkarte</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -12882,17 +12902,17 @@
       <c r="C331" t="inlineStr"/>
       <c r="D331" t="inlineStr">
         <is>
-          <t>.suggestion-box</t>
+          <t>.diary-card-tags</t>
         </is>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>-fx-border-color</t>
+          <t>-fx-fill</t>
         </is>
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>borderColor</t>
+          <t>textColor</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
@@ -12905,7 +12925,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Vorschlagsliste</t>
+          <t>Tagebuchkarte</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -12916,12 +12936,12 @@
       <c r="C332" t="inlineStr"/>
       <c r="D332" t="inlineStr">
         <is>
-          <t>.suggestion-box</t>
+          <t>.diary-card-tags</t>
         </is>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>-fx-border-width</t>
+          <t>-fx-font-style</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
@@ -12936,14 +12956,14 @@
       </c>
       <c r="H332" t="inlineStr">
         <is>
-          <t>"1px"</t>
+          <t>"italic"</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Vorschlagsliste</t>
+          <t>Tagebuchkarte</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -12954,34 +12974,30 @@
       <c r="C333" t="inlineStr"/>
       <c r="D333" t="inlineStr">
         <is>
-          <t>.suggestion-box .label</t>
+          <t>.diary-card-text</t>
         </is>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>-fx-padding</t>
+          <t>-fx-fill</t>
         </is>
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>textColor</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>fest im Code</t>
-        </is>
-      </c>
-      <c r="H333" t="inlineStr">
-        <is>
-          <t>"5 5"</t>
-        </is>
-      </c>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Vorschlagsliste</t>
+          <t>Tagebuchkarte</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -12991,12 +13007,12 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>:highlighted</t>
+          <t>:hover</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>.suggestion-box :highlighted</t>
+          <t>.diary-card:hover</t>
         </is>
       </c>
       <c r="E334" t="inlineStr">
@@ -13006,12 +13022,12 @@
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>menuBarHoverBackground</t>
+          <t>displayTextQuestionBgColor</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>← contrastingShade(menuBarBackground, 20)</t>
+          <t>← displayTextBgColor</t>
         </is>
       </c>
       <c r="H334" t="inlineStr"/>
@@ -13019,28 +13035,28 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Alles (Wurzel)</t>
+          <t>Vorschlagsliste</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>überall</t>
+          <t>Tagebuch</t>
         </is>
       </c>
       <c r="C335" t="inlineStr"/>
       <c r="D335" t="inlineStr">
         <is>
-          <t>.root</t>
+          <t>.suggestion-box</t>
         </is>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>-fx-font-family</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>font</t>
+          <t>menuBarBackground</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
@@ -13048,37 +13064,33 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H335" t="inlineStr">
-        <is>
-          <t>"'" + font.getFamily() + "'"</t>
-        </is>
-      </c>
+      <c r="H335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Alles (Wurzel)</t>
+          <t>Vorschlagsliste</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>überall</t>
+          <t>Tagebuch</t>
         </is>
       </c>
       <c r="C336" t="inlineStr"/>
       <c r="D336" t="inlineStr">
         <is>
-          <t>.root</t>
+          <t>.suggestion-box</t>
         </is>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>-fx-font-size</t>
+          <t>-fx-border-color</t>
         </is>
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t>font</t>
+          <t>borderColor</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -13086,95 +13098,103 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H336" t="inlineStr">
-        <is>
-          <t>font.getSize() + "px"</t>
-        </is>
-      </c>
+      <c r="H336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Bildlaufleiste</t>
+          <t>Vorschlagsliste</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>überall</t>
+          <t>Tagebuch</t>
         </is>
       </c>
       <c r="C337" t="inlineStr"/>
       <c r="D337" t="inlineStr">
         <is>
-          <t>.scroll-bar .increment-arrow, .scroll-bar .decrement-arrow</t>
+          <t>.suggestion-box</t>
         </is>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t>textColor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H337" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>"1px"</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Bildlaufleiste</t>
+          <t>Vorschlagsliste</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>überall</t>
+          <t>Tagebuch</t>
         </is>
       </c>
       <c r="C338" t="inlineStr"/>
       <c r="D338" t="inlineStr">
         <is>
-          <t>.scroll-bar .increment-button, .scroll-bar .decrement-button</t>
+          <t>.suggestion-box .label</t>
         </is>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>menuBarBackground</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H338" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>"5 5"</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Bildlaufleiste</t>
+          <t>Vorschlagsliste</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>überall</t>
-        </is>
-      </c>
-      <c r="C339" t="inlineStr"/>
+          <t>Tagebuch</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>:highlighted</t>
+        </is>
+      </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>.scroll-bar .thumb</t>
+          <t>.suggestion-box :highlighted</t>
         </is>
       </c>
       <c r="E339" t="inlineStr">
@@ -13184,12 +13204,12 @@
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t>activeComponentBgColor</t>
+          <t>menuBarHoverBackground</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>← contrastingShade(menuBarBackground, 20)</t>
         </is>
       </c>
       <c r="H339" t="inlineStr"/>
@@ -13197,7 +13217,7 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Bildlaufleiste</t>
+          <t>Alles (Wurzel)</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
@@ -13205,24 +13225,20 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>:hover</t>
-        </is>
-      </c>
+      <c r="C340" t="inlineStr"/>
       <c r="D340" t="inlineStr">
         <is>
-          <t>.scroll-bar .thumb:hover</t>
+          <t>.root</t>
         </is>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-font-family</t>
         </is>
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>activeComponentHoverColor</t>
+          <t>font</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
@@ -13230,12 +13246,16 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H340" t="inlineStr"/>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>"'" + font.getFamily() + "'"</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Bildlaufleiste</t>
+          <t>Alles (Wurzel)</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
@@ -13246,34 +13266,34 @@
       <c r="C341" t="inlineStr"/>
       <c r="D341" t="inlineStr">
         <is>
-          <t>.scroll-bar .track</t>
+          <t>.root</t>
         </is>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-font-size</t>
         </is>
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>playFieldBackground</t>
+          <t>font</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>← menuBarBackground</t>
+          <t>Pflicht</t>
         </is>
       </c>
       <c r="H341" t="inlineStr">
         <is>
-          <t>UiUtils.contrastingShade(playFieldBackground,10)</t>
+          <t>font.getSize() + "px"</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Eingabefeld</t>
+          <t>Bildlaufleiste</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -13284,34 +13304,30 @@
       <c r="C342" t="inlineStr"/>
       <c r="D342" t="inlineStr">
         <is>
-          <t>.text-field</t>
+          <t>.scroll-bar .increment-arrow, .scroll-bar .decrement-arrow</t>
         </is>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>-fx-alignment</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>textColor</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>fest im Code</t>
-        </is>
-      </c>
-      <c r="H342" t="inlineStr">
-        <is>
-          <t>"center"</t>
-        </is>
-      </c>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Eingabefeld</t>
+          <t>Bildlaufleiste</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
@@ -13322,7 +13338,7 @@
       <c r="C343" t="inlineStr"/>
       <c r="D343" t="inlineStr">
         <is>
-          <t>.text-field</t>
+          <t>.scroll-bar .increment-button, .scroll-bar .decrement-button</t>
         </is>
       </c>
       <c r="E343" t="inlineStr">
@@ -13332,7 +13348,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>activeComponentBgColor</t>
+          <t>menuBarBackground</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -13345,7 +13361,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Eingabefeld</t>
+          <t>Bildlaufleiste</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -13356,17 +13372,17 @@
       <c r="C344" t="inlineStr"/>
       <c r="D344" t="inlineStr">
         <is>
-          <t>.text-field</t>
+          <t>.scroll-bar .thumb</t>
         </is>
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>-fx-background-insets</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>activeComponentBgColor</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -13374,16 +13390,12 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H344" t="inlineStr">
-        <is>
-          <t>borderSmallComponent.width() + "px"</t>
-        </is>
-      </c>
+      <c r="H344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Eingabefeld</t>
+          <t>Bildlaufleiste</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
@@ -13391,20 +13403,24 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C345" t="inlineStr"/>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>:hover</t>
+        </is>
+      </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>.text-field</t>
+          <t>.scroll-bar .thumb:hover</t>
         </is>
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>-fx-background-radius</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>activeComponentHoverColor</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -13412,16 +13428,12 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H345" t="inlineStr">
-        <is>
-          <t>borderSmallComponent.arc() + "px"</t>
-        </is>
-      </c>
+      <c r="H345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Eingabefeld</t>
+          <t>Bildlaufleiste</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -13432,27 +13444,27 @@
       <c r="C346" t="inlineStr"/>
       <c r="D346" t="inlineStr">
         <is>
-          <t>.text-field</t>
+          <t>.scroll-bar .track</t>
         </is>
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>-fx-border-color</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>playFieldBackground</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>← menuBarBackground</t>
         </is>
       </c>
       <c r="H346" t="inlineStr">
         <is>
-          <t>borderSmallComponent.color()</t>
+          <t>UiUtils.contrastingShade(playFieldBackground,10)</t>
         </is>
       </c>
     </row>
@@ -13475,22 +13487,22 @@
       </c>
       <c r="E347" t="inlineStr">
         <is>
-          <t>-fx-border-radius</t>
+          <t>-fx-alignment</t>
         </is>
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>fest im Code</t>
         </is>
       </c>
       <c r="H347" t="inlineStr">
         <is>
-          <t>borderSmallComponent.arc() + "px"</t>
+          <t>"center"</t>
         </is>
       </c>
     </row>
@@ -13513,12 +13525,12 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>-fx-border-width</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>activeComponentBgColor</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -13526,11 +13538,7 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H348" t="inlineStr">
-        <is>
-          <t>borderSmallComponent.width() + "px"</t>
-        </is>
-      </c>
+      <c r="H348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -13551,20 +13559,24 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>-fx-effect</t>
+          <t>-fx-background-insets</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t>componentShadow</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>entfällt</t>
-        </is>
-      </c>
-      <c r="H349" t="inlineStr"/>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>borderSmallComponent.width() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -13585,7 +13597,7 @@
       </c>
       <c r="E350" t="inlineStr">
         <is>
-          <t>-fx-padding</t>
+          <t>-fx-background-radius</t>
         </is>
       </c>
       <c r="F350" t="inlineStr">
@@ -13600,7 +13612,7 @@
       </c>
       <c r="H350" t="inlineStr">
         <is>
-          <t>paddingCss</t>
+          <t>borderSmallComponent.arc() + "px"</t>
         </is>
       </c>
     </row>
@@ -13623,20 +13635,24 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>-fx-text-fill</t>
+          <t>-fx-border-color</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t>textActiveComponentColor</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>← textColor</t>
-        </is>
-      </c>
-      <c r="H351" t="inlineStr"/>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>borderSmallComponent.color()</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -13649,24 +13665,20 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C352" t="inlineStr">
-        <is>
-          <t>:disabled</t>
-        </is>
-      </c>
+      <c r="C352" t="inlineStr"/>
       <c r="D352" t="inlineStr">
         <is>
-          <t>.text-field:disabled</t>
+          <t>.text-field</t>
         </is>
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-border-radius</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t>disabledComponentBgColor</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
@@ -13674,7 +13686,11 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H352" t="inlineStr"/>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>borderSmallComponent.arc() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -13687,19 +13703,15 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C353" t="inlineStr">
-        <is>
-          <t>:disabled</t>
-        </is>
-      </c>
+      <c r="C353" t="inlineStr"/>
       <c r="D353" t="inlineStr">
         <is>
-          <t>.text-field:disabled</t>
+          <t>.text-field</t>
         </is>
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>-fx-border-color</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
@@ -13714,7 +13726,7 @@
       </c>
       <c r="H353" t="inlineStr">
         <is>
-          <t>borderSmallComponent.disabledColor()</t>
+          <t>borderSmallComponent.width() + "px"</t>
         </is>
       </c>
     </row>
@@ -13729,36 +13741,28 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C354" t="inlineStr">
-        <is>
-          <t>:disabled</t>
-        </is>
-      </c>
+      <c r="C354" t="inlineStr"/>
       <c r="D354" t="inlineStr">
         <is>
-          <t>.text-field:disabled</t>
+          <t>.text-field</t>
         </is>
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>-fx-font-weight</t>
+          <t>-fx-effect</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>componentShadow</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>fest im Code</t>
-        </is>
-      </c>
-      <c r="H354" t="inlineStr">
-        <is>
-          <t>"bold"</t>
-        </is>
-      </c>
+          <t>entfällt</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -13771,34 +13775,30 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C355" t="inlineStr">
-        <is>
-          <t>:disabled</t>
-        </is>
-      </c>
+      <c r="C355" t="inlineStr"/>
       <c r="D355" t="inlineStr">
         <is>
-          <t>.text-field:disabled</t>
+          <t>.text-field</t>
         </is>
       </c>
       <c r="E355" t="inlineStr">
         <is>
-          <t>-fx-opacity</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>fest im Code</t>
+          <t>Pflicht</t>
         </is>
       </c>
       <c r="H355" t="inlineStr">
         <is>
-          <t>"1.0"</t>
+          <t>paddingCss</t>
         </is>
       </c>
     </row>
@@ -13813,14 +13813,10 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr">
-        <is>
-          <t>:disabled</t>
-        </is>
-      </c>
+      <c r="C356" t="inlineStr"/>
       <c r="D356" t="inlineStr">
         <is>
-          <t>.text-field:disabled</t>
+          <t>.text-field</t>
         </is>
       </c>
       <c r="E356" t="inlineStr">
@@ -13830,12 +13826,12 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t>incorrectTextColor</t>
+          <t>textActiveComponentColor</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>← textColor</t>
         </is>
       </c>
       <c r="H356" t="inlineStr"/>
@@ -13853,27 +13849,27 @@
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>:focused</t>
+          <t>:disabled</t>
         </is>
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>.text-field:focused</t>
+          <t>.text-field:disabled</t>
         </is>
       </c>
       <c r="E357" t="inlineStr">
         <is>
-          <t>-fx-background-insets</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t>activeBorderWidth</t>
+          <t>disabledComponentBgColor</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Pflicht</t>
         </is>
       </c>
       <c r="H357" t="inlineStr"/>
@@ -13891,12 +13887,12 @@
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>:focused</t>
+          <t>:disabled</t>
         </is>
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>.text-field:focused</t>
+          <t>.text-field:disabled</t>
         </is>
       </c>
       <c r="E358" t="inlineStr">
@@ -13906,15 +13902,19 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t>activeBorderColor</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>entfällt</t>
-        </is>
-      </c>
-      <c r="H358" t="inlineStr"/>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>borderSmallComponent.disabledColor()</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -13929,30 +13929,34 @@
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>:focused</t>
+          <t>:disabled</t>
         </is>
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>.text-field:focused</t>
+          <t>.text-field:disabled</t>
         </is>
       </c>
       <c r="E359" t="inlineStr">
         <is>
-          <t>-fx-border-width</t>
+          <t>-fx-font-weight</t>
         </is>
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t>activeBorderWidth</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="H359" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>"bold"</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -13967,35 +13971,39 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>:invalid-query</t>
+          <t>:disabled</t>
         </is>
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>.text-field:invalid-query</t>
+          <t>.text-field:disabled</t>
         </is>
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>-fx-text-fill</t>
+          <t>-fx-opacity</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t>incorrectTextColor</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H360" t="inlineStr"/>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>"1.0"</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>Jeder Text</t>
+          <t>Eingabefeld</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
@@ -14003,20 +14011,24 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr"/>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>:disabled</t>
+        </is>
+      </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>.text</t>
+          <t>.text-field:disabled</t>
         </is>
       </c>
       <c r="E361" t="inlineStr">
         <is>
-          <t>-fx-fill</t>
+          <t>-fx-text-fill</t>
         </is>
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t>textColor</t>
+          <t>incorrectTextColor</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -14029,7 +14041,7 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>Knopf</t>
+          <t>Eingabefeld</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
@@ -14037,25 +14049,29 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C362" t="inlineStr"/>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>.button .text, .date-picker .arrow-button .text</t>
+          <t>.text-field:focused</t>
         </is>
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>-fx-fill</t>
+          <t>-fx-background-insets</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t>textActiveComponentColor</t>
+          <t>activeBorderWidth</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>← textColor</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H362" t="inlineStr"/>
@@ -14063,7 +14079,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Knopf</t>
+          <t>Eingabefeld</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
@@ -14071,25 +14087,29 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C363" t="inlineStr"/>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
+          <t>.text-field:focused</t>
         </is>
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-border-color</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t>activeComponentBgColor</t>
+          <t>activeBorderColor</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>entfällt</t>
         </is>
       </c>
       <c r="H363" t="inlineStr"/>
@@ -14097,7 +14117,7 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>Knopf</t>
+          <t>Eingabefeld</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
@@ -14105,37 +14125,37 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C364" t="inlineStr"/>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
+          <t>.text-field:focused</t>
         </is>
       </c>
       <c r="E364" t="inlineStr">
         <is>
-          <t>-fx-background-insets</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>activeBorderWidth</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H364" t="inlineStr">
-        <is>
-          <t>borderSmallComponent.width() + "px"</t>
-        </is>
-      </c>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>Knopf</t>
+          <t>Eingabefeld</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
@@ -14143,20 +14163,24 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C365" t="inlineStr"/>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>:invalid-query</t>
+        </is>
+      </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
+          <t>.text-field:invalid-query</t>
         </is>
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>-fx-background-radius</t>
+          <t>-fx-text-fill</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>incorrectTextColor</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
@@ -14164,16 +14188,12 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H365" t="inlineStr">
-        <is>
-          <t>borderSmallComponent.arc() + "px"</t>
-        </is>
-      </c>
+      <c r="H365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>Knopf</t>
+          <t>Jeder Text</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
@@ -14184,17 +14204,17 @@
       <c r="C366" t="inlineStr"/>
       <c r="D366" t="inlineStr">
         <is>
-          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
+          <t>.text</t>
         </is>
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>-fx-border-color</t>
+          <t>-fx-fill</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>textColor</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -14202,11 +14222,7 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H366" t="inlineStr">
-        <is>
-          <t>borderSmallComponent.color()</t>
-        </is>
-      </c>
+      <c r="H366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -14222,29 +14238,25 @@
       <c r="C367" t="inlineStr"/>
       <c r="D367" t="inlineStr">
         <is>
-          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
+          <t>.button .text, .date-picker .arrow-button .text</t>
         </is>
       </c>
       <c r="E367" t="inlineStr">
         <is>
-          <t>-fx-border-radius</t>
+          <t>-fx-fill</t>
         </is>
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>textActiveComponentColor</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H367" t="inlineStr">
-        <is>
-          <t>borderSmallComponent.arc() + "px"</t>
-        </is>
-      </c>
+          <t>← textColor</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -14265,12 +14277,12 @@
       </c>
       <c r="E368" t="inlineStr">
         <is>
-          <t>-fx-border-width</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F368" t="inlineStr">
         <is>
-          <t>borderSmallComponent</t>
+          <t>activeComponentBgColor</t>
         </is>
       </c>
       <c r="G368" t="inlineStr">
@@ -14278,11 +14290,7 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H368" t="inlineStr">
-        <is>
-          <t>borderSmallComponent.width() + "px"</t>
-        </is>
-      </c>
+      <c r="H368" t="inlineStr"/>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
@@ -14303,20 +14311,24 @@
       </c>
       <c r="E369" t="inlineStr">
         <is>
-          <t>-fx-effect</t>
+          <t>-fx-background-insets</t>
         </is>
       </c>
       <c r="F369" t="inlineStr">
         <is>
-          <t>componentShadow</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G369" t="inlineStr">
         <is>
-          <t>entfällt</t>
-        </is>
-      </c>
-      <c r="H369" t="inlineStr"/>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>borderSmallComponent.width() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -14329,24 +14341,20 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C370" t="inlineStr">
-        <is>
-          <t>:hover, :hover</t>
-        </is>
-      </c>
+      <c r="C370" t="inlineStr"/>
       <c r="D370" t="inlineStr">
         <is>
-          <t>.button:hover, .date-picker .arrow-button:hover</t>
+          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
         </is>
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-background-radius</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
         <is>
-          <t>activeComponentHoverColor</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G370" t="inlineStr">
@@ -14354,7 +14362,11 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H370" t="inlineStr"/>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>borderSmallComponent.arc() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -14367,24 +14379,20 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C371" t="inlineStr">
-        <is>
-          <t>:pressed, :pressed</t>
-        </is>
-      </c>
+      <c r="C371" t="inlineStr"/>
       <c r="D371" t="inlineStr">
         <is>
-          <t>.button:pressed, .date-picker .arrow-button:pressed</t>
+          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
         </is>
       </c>
       <c r="E371" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-border-color</t>
         </is>
       </c>
       <c r="F371" t="inlineStr">
         <is>
-          <t>activeComponentHoverColor</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G371" t="inlineStr">
@@ -14394,14 +14402,14 @@
       </c>
       <c r="H371" t="inlineStr">
         <is>
-          <t>UiUtils.contrastingShade(activeComponentHoverColor, 8)</t>
+          <t>borderSmallComponent.color()</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>Menü</t>
+          <t>Knopf</t>
         </is>
       </c>
       <c r="B372" t="inlineStr">
@@ -14412,17 +14420,17 @@
       <c r="C372" t="inlineStr"/>
       <c r="D372" t="inlineStr">
         <is>
-          <t>.context-menu</t>
+          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
         </is>
       </c>
       <c r="E372" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-border-radius</t>
         </is>
       </c>
       <c r="F372" t="inlineStr">
         <is>
-          <t>menuBarBackground</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G372" t="inlineStr">
@@ -14430,12 +14438,16 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H372" t="inlineStr"/>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>borderSmallComponent.arc() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>Menü</t>
+          <t>Knopf</t>
         </is>
       </c>
       <c r="B373" t="inlineStr">
@@ -14446,17 +14458,17 @@
       <c r="C373" t="inlineStr"/>
       <c r="D373" t="inlineStr">
         <is>
-          <t>.context-menu</t>
+          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
         </is>
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>-fx-border-color</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
         <is>
-          <t>thinBorderColor</t>
+          <t>borderSmallComponent</t>
         </is>
       </c>
       <c r="G373" t="inlineStr">
@@ -14464,12 +14476,16 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H373" t="inlineStr"/>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>borderSmallComponent.width() + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>Menü</t>
+          <t>Knopf</t>
         </is>
       </c>
       <c r="B374" t="inlineStr">
@@ -14480,34 +14496,30 @@
       <c r="C374" t="inlineStr"/>
       <c r="D374" t="inlineStr">
         <is>
-          <t>.context-menu</t>
+          <t>.button, .date-picker .arrow-button, .spinner .increment-arrow-button, .spinner .decrement-arrow-button</t>
         </is>
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>-fx-border-width</t>
+          <t>-fx-effect</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
         <is>
-          <t>thinBorderWidth</t>
+          <t>componentShadow</t>
         </is>
       </c>
       <c r="G374" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H374" t="inlineStr">
-        <is>
-          <t>thinBorderWidth + "px"</t>
-        </is>
-      </c>
+          <t>entfällt</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>Menü</t>
+          <t>Knopf</t>
         </is>
       </c>
       <c r="B375" t="inlineStr">
@@ -14515,10 +14527,14 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C375" t="inlineStr"/>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>:hover, :hover</t>
+        </is>
+      </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>.menu-bar</t>
+          <t>.button:hover, .date-picker .arrow-button:hover</t>
         </is>
       </c>
       <c r="E375" t="inlineStr">
@@ -14528,7 +14544,7 @@
       </c>
       <c r="F375" t="inlineStr">
         <is>
-          <t>menuBarBackground</t>
+          <t>activeComponentHoverColor</t>
         </is>
       </c>
       <c r="G375" t="inlineStr">
@@ -14541,7 +14557,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>Menü</t>
+          <t>Knopf</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
@@ -14549,28 +14565,36 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C376" t="inlineStr"/>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>:pressed, :pressed</t>
+        </is>
+      </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>.menu-button</t>
+          <t>.button:pressed, .date-picker .arrow-button:pressed</t>
         </is>
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>-fx-padding</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>menuButtonPadding</t>
+          <t>activeComponentHoverColor</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>← font × 0,3 / 0,4</t>
-        </is>
-      </c>
-      <c r="H376" t="inlineStr"/>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>UiUtils.contrastingShade(activeComponentHoverColor, 8)</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
@@ -14586,17 +14610,17 @@
       <c r="C377" t="inlineStr"/>
       <c r="D377" t="inlineStr">
         <is>
-          <t>.menu-item</t>
+          <t>.context-menu</t>
         </is>
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>-fx-font-family</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t>font</t>
+          <t>menuBarBackground</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
@@ -14604,11 +14628,7 @@
           <t>Pflicht</t>
         </is>
       </c>
-      <c r="H377" t="inlineStr">
-        <is>
-          <t>"'" + font.getFamily() + "'"</t>
-        </is>
-      </c>
+      <c r="H377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -14624,22 +14644,22 @@
       <c r="C378" t="inlineStr"/>
       <c r="D378" t="inlineStr">
         <is>
-          <t>.menu-item</t>
+          <t>.context-menu</t>
         </is>
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t>-fx-padding</t>
+          <t>-fx-border-color</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t>menuItemPadding</t>
+          <t>thinBorderColor</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t>← font × 0,1 / 0,5</t>
+          <t>Pflicht</t>
         </is>
       </c>
       <c r="H378" t="inlineStr"/>
@@ -14655,32 +14675,32 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C379" t="inlineStr">
-        <is>
-          <t>:disabled</t>
-        </is>
-      </c>
+      <c r="C379" t="inlineStr"/>
       <c r="D379" t="inlineStr">
         <is>
-          <t>.menu-item:disabled .label</t>
+          <t>.context-menu</t>
         </is>
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t>-fx-text-fill</t>
+          <t>-fx-border-width</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t>textColor</t>
+          <t>thinBorderWidth</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H379" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>thinBorderWidth + "px"</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -14693,14 +14713,10 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C380" t="inlineStr">
-        <is>
-          <t>:disabled, :hover</t>
-        </is>
-      </c>
+      <c r="C380" t="inlineStr"/>
       <c r="D380" t="inlineStr">
         <is>
-          <t>.menu-item:disabled:hover</t>
+          <t>.menu-bar</t>
         </is>
       </c>
       <c r="E380" t="inlineStr">
@@ -14710,19 +14726,15 @@
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>menuBarBackground</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
         <is>
-          <t>fest im Code</t>
-        </is>
-      </c>
-      <c r="H380" t="inlineStr">
-        <is>
-          <t>"transparent"</t>
-        </is>
-      </c>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr"/>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
@@ -14735,29 +14747,25 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C381" t="inlineStr">
-        <is>
-          <t>:focused</t>
-        </is>
-      </c>
+      <c r="C381" t="inlineStr"/>
       <c r="D381" t="inlineStr">
         <is>
-          <t>.menu-item:focused</t>
+          <t>.menu-button</t>
         </is>
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t>menuBarHoverBackground</t>
+          <t>menuButtonPadding</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
         <is>
-          <t>← contrastingShade(menuBarBackground, 20)</t>
+          <t>← font × 0,3 / 0,4</t>
         </is>
       </c>
       <c r="H381" t="inlineStr"/>
@@ -14773,32 +14781,32 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C382" t="inlineStr">
-        <is>
-          <t>:hover</t>
-        </is>
-      </c>
+      <c r="C382" t="inlineStr"/>
       <c r="D382" t="inlineStr">
         <is>
-          <t>.menu-item:hover</t>
+          <t>.menu-item</t>
         </is>
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-font-family</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t>menuBarHoverBackground</t>
+          <t>font</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
         <is>
-          <t>← contrastingShade(menuBarBackground, 20)</t>
-        </is>
-      </c>
-      <c r="H382" t="inlineStr"/>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>"'" + font.getFamily() + "'"</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
@@ -14811,29 +14819,25 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C383" t="inlineStr">
-        <is>
-          <t>:hover</t>
-        </is>
-      </c>
+      <c r="C383" t="inlineStr"/>
       <c r="D383" t="inlineStr">
         <is>
-          <t>.menu:hover</t>
+          <t>.menu-item</t>
         </is>
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-padding</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t>menuBarHoverBackground</t>
+          <t>menuItemPadding</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
         <is>
-          <t>← contrastingShade(menuBarBackground, 20)</t>
+          <t>← font × 0,1 / 0,5</t>
         </is>
       </c>
       <c r="H383" t="inlineStr"/>
@@ -14851,27 +14855,27 @@
       </c>
       <c r="C384" t="inlineStr">
         <is>
-          <t>:showing</t>
+          <t>:disabled</t>
         </is>
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>.menu:showing</t>
+          <t>.menu-item:disabled .label</t>
         </is>
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>-fx-background-color</t>
+          <t>-fx-text-fill</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t>menuBarHoverBackground</t>
+          <t>textColor</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
         <is>
-          <t>← contrastingShade(menuBarBackground, 20)</t>
+          <t>Pflicht</t>
         </is>
       </c>
       <c r="H384" t="inlineStr"/>
@@ -14887,15 +14891,19 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C385" t="inlineStr"/>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>:disabled, :hover</t>
+        </is>
+      </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>.my-spacer</t>
+          <t>.menu-item:disabled:hover</t>
         </is>
       </c>
       <c r="E385" t="inlineStr">
         <is>
-          <t>-fx-opacity</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
@@ -14910,7 +14918,7 @@
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t>"0"</t>
+          <t>"transparent"</t>
         </is>
       </c>
     </row>
@@ -14925,37 +14933,37 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C386" t="inlineStr"/>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>:focused</t>
+        </is>
+      </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>.my-spacer</t>
+          <t>.menu-item:focused</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>-fx-pref-height</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t>font</t>
+          <t>menuBarHoverBackground</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
         <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H386" t="inlineStr">
-        <is>
-          <t>"" + font.getSize() * 0.3 + "px"</t>
-        </is>
-      </c>
+          <t>← contrastingShade(menuBarBackground, 20)</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr"/>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>Titelleiste des Hauptfensters</t>
+          <t>Menü</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
@@ -14963,10 +14971,14 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C387" t="inlineStr"/>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>:hover</t>
+        </is>
+      </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>.my-header-bar</t>
+          <t>.menu-item:hover</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -14976,12 +14988,12 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>menuBarBackground</t>
+          <t>menuBarHoverBackground</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>← contrastingShade(menuBarBackground, 20)</t>
         </is>
       </c>
       <c r="H387" t="inlineStr"/>
@@ -14989,7 +15001,7 @@
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>Titelleiste des Hauptfensters</t>
+          <t>Menü</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -14997,25 +15009,29 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C388" t="inlineStr"/>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>:hover</t>
+        </is>
+      </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>.my-header-bar</t>
+          <t>.menu:hover</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
         <is>
-          <t>-fx-border-color</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>thinBorderColor</t>
+          <t>menuBarHoverBackground</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>Pflicht</t>
+          <t>← contrastingShade(menuBarBackground, 20)</t>
         </is>
       </c>
       <c r="H388" t="inlineStr"/>
@@ -15023,7 +15039,7 @@
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>Titelleiste des Hauptfensters</t>
+          <t>Menü</t>
         </is>
       </c>
       <c r="B389" t="inlineStr">
@@ -15031,37 +15047,37 @@
           <t>überall</t>
         </is>
       </c>
-      <c r="C389" t="inlineStr"/>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>:showing</t>
+        </is>
+      </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>.my-header-bar</t>
+          <t>.menu:showing</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>-fx-border-width</t>
+          <t>-fx-background-color</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>menuBarHoverBackground</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
         <is>
-          <t>fest im Code</t>
-        </is>
-      </c>
-      <c r="H389" t="inlineStr">
-        <is>
-          <t>"0 0 1 0"</t>
-        </is>
-      </c>
+          <t>← contrastingShade(menuBarBackground, 20)</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr"/>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>Titelleiste des Hauptfensters</t>
+          <t>Menü</t>
         </is>
       </c>
       <c r="B390" t="inlineStr">
@@ -15072,32 +15088,214 @@
       <c r="C390" t="inlineStr"/>
       <c r="D390" t="inlineStr">
         <is>
+          <t>.my-spacer</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>-fx-opacity</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>"0"</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Menü</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>überall</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr"/>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>.my-spacer</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>-fx-pref-height</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>font</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>"" + font.getSize() * 0.3 + "px"</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Titelleiste des Hauptfensters</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>überall</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr"/>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>.my-header-bar</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>-fx-background-color</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>menuBarBackground</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Titelleiste des Hauptfensters</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>überall</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr"/>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>.my-header-bar</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>-fx-border-color</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>thinBorderColor</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Titelleiste des Hauptfensters</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>überall</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr"/>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>.my-header-bar</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>-fx-border-width</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>fest im Code</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>"0 0 1 0"</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Titelleiste des Hauptfensters</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>überall</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr"/>
+      <c r="D395" t="inlineStr">
+        <is>
           <t>.my-header-leading</t>
         </is>
       </c>
-      <c r="E390" t="inlineStr">
+      <c r="E395" t="inlineStr">
         <is>
           <t>-fx-padding</t>
         </is>
       </c>
-      <c r="F390" t="inlineStr">
+      <c r="F395" t="inlineStr">
         <is>
           <t>font</t>
         </is>
       </c>
-      <c r="G390" t="inlineStr">
-        <is>
-          <t>Pflicht</t>
-        </is>
-      </c>
-      <c r="H390" t="inlineStr">
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>Pflicht</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
         <is>
           <t>"0 0 0 " + (font.getSize() * 0.5) + "px"</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H390"/>
+  <autoFilter ref="A1:H395"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>